<commit_message>
feat: add EU/Non-EU region indicator to transactions view and modal
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/research/DPD_FX SWAP_202601.xlsx
+++ b/research/DPD_FX SWAP_202601.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\x200709\Desktop\WSS\CURSOR\Pliki źródłowe\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lukas\milleVAT\milleVAT\research\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{901F11ED-483B-4527-A609-C494EE680747}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{680F398A-225D-450B-8DE3-155C6FFE2160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -939,7 +939,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:W215"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
     <col min="2" max="3" width="15" customWidth="1"/>
@@ -960,7 +960,7 @@
     <col min="23" max="23" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1031,7 +1031,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>115</v>
       </c>
@@ -1102,7 +1102,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>115</v>
       </c>
@@ -1173,7 +1173,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>115</v>
       </c>
@@ -1244,7 +1244,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>115</v>
       </c>
@@ -1315,7 +1315,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>115</v>
       </c>
@@ -1386,7 +1386,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>115</v>
       </c>
@@ -1457,7 +1457,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>115</v>
       </c>
@@ -1528,7 +1528,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>115</v>
       </c>
@@ -1599,7 +1599,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>115</v>
       </c>
@@ -1670,7 +1670,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>115</v>
       </c>
@@ -1741,7 +1741,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>115</v>
       </c>
@@ -1812,7 +1812,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>115</v>
       </c>
@@ -1883,7 +1883,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>115</v>
       </c>
@@ -1954,7 +1954,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>115</v>
       </c>
@@ -2025,7 +2025,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>115</v>
       </c>
@@ -2096,7 +2096,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>115</v>
       </c>
@@ -2167,7 +2167,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>115</v>
       </c>
@@ -2238,7 +2238,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>115</v>
       </c>
@@ -2309,7 +2309,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>115</v>
       </c>
@@ -2380,7 +2380,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>115</v>
       </c>
@@ -2451,7 +2451,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>115</v>
       </c>
@@ -2522,7 +2522,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>115</v>
       </c>
@@ -2593,7 +2593,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>115</v>
       </c>
@@ -2664,7 +2664,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>115</v>
       </c>
@@ -2735,7 +2735,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>115</v>
       </c>
@@ -2806,7 +2806,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>115</v>
       </c>
@@ -2877,7 +2877,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>115</v>
       </c>
@@ -2948,7 +2948,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>115</v>
       </c>
@@ -3019,7 +3019,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>115</v>
       </c>
@@ -3090,7 +3090,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>115</v>
       </c>
@@ -3161,7 +3161,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>115</v>
       </c>
@@ -3232,7 +3232,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>115</v>
       </c>
@@ -3303,7 +3303,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>115</v>
       </c>
@@ -3374,7 +3374,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="36" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>115</v>
       </c>
@@ -3445,7 +3445,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="37" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>115</v>
       </c>
@@ -3516,7 +3516,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="38" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>115</v>
       </c>
@@ -3587,7 +3587,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="39" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>115</v>
       </c>
@@ -3658,7 +3658,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="40" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>115</v>
       </c>
@@ -3729,7 +3729,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="41" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>115</v>
       </c>
@@ -3800,7 +3800,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="42" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>115</v>
       </c>
@@ -3871,7 +3871,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="43" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>115</v>
       </c>
@@ -3942,7 +3942,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="44" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>115</v>
       </c>
@@ -4013,7 +4013,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="45" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>115</v>
       </c>
@@ -4084,7 +4084,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="46" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>115</v>
       </c>
@@ -4155,7 +4155,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="47" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>115</v>
       </c>
@@ -4226,7 +4226,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="48" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>115</v>
       </c>
@@ -4297,7 +4297,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="49" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>115</v>
       </c>
@@ -4368,7 +4368,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="50" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>115</v>
       </c>
@@ -4439,7 +4439,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="51" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>115</v>
       </c>
@@ -4510,7 +4510,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="52" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>115</v>
       </c>
@@ -4581,7 +4581,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="53" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>115</v>
       </c>
@@ -4652,7 +4652,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="54" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>115</v>
       </c>
@@ -4723,7 +4723,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="55" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>115</v>
       </c>
@@ -4794,7 +4794,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="56" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>115</v>
       </c>
@@ -4865,7 +4865,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="57" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>115</v>
       </c>
@@ -4936,7 +4936,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="58" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>115</v>
       </c>
@@ -5007,7 +5007,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="59" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>115</v>
       </c>
@@ -5078,7 +5078,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="60" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>115</v>
       </c>
@@ -5149,7 +5149,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="61" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>115</v>
       </c>
@@ -5220,7 +5220,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="62" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>115</v>
       </c>
@@ -5291,7 +5291,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="63" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>115</v>
       </c>
@@ -5362,7 +5362,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="64" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>115</v>
       </c>
@@ -5433,7 +5433,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="65" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>115</v>
       </c>
@@ -5504,7 +5504,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="66" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>115</v>
       </c>
@@ -5575,7 +5575,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="67" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>115</v>
       </c>
@@ -5646,7 +5646,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="68" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>115</v>
       </c>
@@ -5717,7 +5717,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="69" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>115</v>
       </c>
@@ -5788,7 +5788,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="70" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>115</v>
       </c>
@@ -5859,7 +5859,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="71" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>115</v>
       </c>
@@ -5930,7 +5930,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="72" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>115</v>
       </c>
@@ -6001,7 +6001,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="73" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>115</v>
       </c>
@@ -6072,7 +6072,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="74" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>115</v>
       </c>
@@ -6143,7 +6143,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="75" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
         <v>115</v>
       </c>
@@ -6214,7 +6214,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="76" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
         <v>115</v>
       </c>
@@ -6285,7 +6285,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="77" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
         <v>115</v>
       </c>
@@ -6356,7 +6356,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="78" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
         <v>115</v>
       </c>
@@ -6427,7 +6427,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="79" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
         <v>115</v>
       </c>
@@ -6498,7 +6498,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="80" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
         <v>115</v>
       </c>
@@ -6569,7 +6569,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="81" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
         <v>115</v>
       </c>
@@ -6640,7 +6640,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="82" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
         <v>115</v>
       </c>
@@ -6711,7 +6711,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="83" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
         <v>115</v>
       </c>
@@ -6782,7 +6782,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="84" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
         <v>115</v>
       </c>
@@ -6853,7 +6853,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="85" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
         <v>115</v>
       </c>
@@ -6924,7 +6924,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="86" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
         <v>115</v>
       </c>
@@ -6995,7 +6995,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="87" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
         <v>115</v>
       </c>
@@ -7066,7 +7066,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="88" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
         <v>115</v>
       </c>
@@ -7137,7 +7137,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="89" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
         <v>115</v>
       </c>
@@ -7208,7 +7208,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="90" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
         <v>115</v>
       </c>
@@ -7279,7 +7279,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="91" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
         <v>115</v>
       </c>
@@ -7350,7 +7350,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="92" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
         <v>115</v>
       </c>
@@ -7421,7 +7421,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="93" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A93" s="2" t="s">
         <v>115</v>
       </c>
@@ -7492,7 +7492,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="94" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A94" s="2" t="s">
         <v>115</v>
       </c>
@@ -7563,7 +7563,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="95" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A95" s="2" t="s">
         <v>115</v>
       </c>
@@ -7634,7 +7634,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="96" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A96" s="2" t="s">
         <v>115</v>
       </c>
@@ -7705,7 +7705,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="97" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A97" s="2" t="s">
         <v>115</v>
       </c>
@@ -7776,7 +7776,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="98" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
         <v>115</v>
       </c>
@@ -7847,7 +7847,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="99" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A99" s="2" t="s">
         <v>115</v>
       </c>
@@ -7918,7 +7918,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="100" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A100" s="2" t="s">
         <v>115</v>
       </c>
@@ -7989,7 +7989,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="101" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
         <v>115</v>
       </c>
@@ -8060,7 +8060,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="102" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A102" s="2" t="s">
         <v>115</v>
       </c>
@@ -8131,7 +8131,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="103" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A103" s="2" t="s">
         <v>115</v>
       </c>
@@ -8202,7 +8202,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="104" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A104" s="2" t="s">
         <v>115</v>
       </c>
@@ -8273,7 +8273,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="105" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A105" s="2" t="s">
         <v>115</v>
       </c>
@@ -8344,7 +8344,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="106" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A106" s="2" t="s">
         <v>115</v>
       </c>
@@ -8415,7 +8415,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="107" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
         <v>115</v>
       </c>
@@ -8486,7 +8486,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="108" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A108" s="2" t="s">
         <v>115</v>
       </c>
@@ -8557,7 +8557,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="109" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A109" s="2" t="s">
         <v>115</v>
       </c>
@@ -8628,7 +8628,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="110" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A110" s="2" t="s">
         <v>115</v>
       </c>
@@ -8699,7 +8699,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="111" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A111" s="2" t="s">
         <v>115</v>
       </c>
@@ -8770,7 +8770,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="112" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A112" s="2" t="s">
         <v>115</v>
       </c>
@@ -8841,7 +8841,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="113" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A113" s="2" t="s">
         <v>115</v>
       </c>
@@ -8912,7 +8912,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="114" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A114" s="2" t="s">
         <v>115</v>
       </c>
@@ -8983,7 +8983,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="115" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A115" s="2" t="s">
         <v>115</v>
       </c>
@@ -9054,7 +9054,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="116" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A116" s="2" t="s">
         <v>115</v>
       </c>
@@ -9125,7 +9125,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="117" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A117" s="2" t="s">
         <v>115</v>
       </c>
@@ -9196,7 +9196,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="118" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A118" s="2" t="s">
         <v>115</v>
       </c>
@@ -9267,7 +9267,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="119" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A119" s="2" t="s">
         <v>115</v>
       </c>
@@ -9338,7 +9338,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="120" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A120" s="2" t="s">
         <v>115</v>
       </c>
@@ -9409,7 +9409,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="121" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A121" s="2" t="s">
         <v>115</v>
       </c>
@@ -9480,7 +9480,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="122" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A122" s="2" t="s">
         <v>115</v>
       </c>
@@ -9551,7 +9551,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="123" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A123" s="2" t="s">
         <v>115</v>
       </c>
@@ -9622,7 +9622,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="124" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A124" s="2" t="s">
         <v>115</v>
       </c>
@@ -9693,7 +9693,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="125" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A125" s="2" t="s">
         <v>115</v>
       </c>
@@ -9764,7 +9764,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="126" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A126" s="2" t="s">
         <v>115</v>
       </c>
@@ -9835,7 +9835,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="127" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A127" s="2" t="s">
         <v>115</v>
       </c>
@@ -9906,7 +9906,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="128" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A128" s="2" t="s">
         <v>115</v>
       </c>
@@ -9977,7 +9977,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="129" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A129" s="2" t="s">
         <v>115</v>
       </c>
@@ -10048,7 +10048,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="130" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A130" s="2" t="s">
         <v>115</v>
       </c>
@@ -10119,7 +10119,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="131" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A131" s="2" t="s">
         <v>115</v>
       </c>
@@ -10190,7 +10190,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="132" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A132" s="2" t="s">
         <v>115</v>
       </c>
@@ -10261,7 +10261,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="133" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A133" s="2" t="s">
         <v>115</v>
       </c>
@@ -10332,7 +10332,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="134" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A134" s="2" t="s">
         <v>115</v>
       </c>
@@ -10403,7 +10403,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="135" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A135" s="2" t="s">
         <v>115</v>
       </c>
@@ -10474,7 +10474,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="136" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A136" s="2" t="s">
         <v>115</v>
       </c>
@@ -10545,7 +10545,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="137" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A137" s="2" t="s">
         <v>115</v>
       </c>
@@ -10616,7 +10616,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="138" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A138" s="2" t="s">
         <v>115</v>
       </c>
@@ -10687,7 +10687,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="139" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A139" s="2" t="s">
         <v>115</v>
       </c>
@@ -10758,7 +10758,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="140" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A140" s="2" t="s">
         <v>115</v>
       </c>
@@ -10829,7 +10829,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="141" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A141" s="2" t="s">
         <v>115</v>
       </c>
@@ -10900,7 +10900,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="142" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A142" s="2" t="s">
         <v>115</v>
       </c>
@@ -10971,7 +10971,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="143" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A143" s="2" t="s">
         <v>115</v>
       </c>
@@ -11042,7 +11042,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="144" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A144" s="2" t="s">
         <v>115</v>
       </c>
@@ -11113,7 +11113,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="145" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A145" s="2" t="s">
         <v>115</v>
       </c>
@@ -11184,7 +11184,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="146" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A146" s="2" t="s">
         <v>115</v>
       </c>
@@ -11255,7 +11255,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="147" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A147" s="2" t="s">
         <v>115</v>
       </c>
@@ -11326,7 +11326,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="148" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A148" s="2" t="s">
         <v>115</v>
       </c>
@@ -11397,7 +11397,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="149" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A149" s="2" t="s">
         <v>115</v>
       </c>
@@ -11468,7 +11468,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="150" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A150" s="2" t="s">
         <v>115</v>
       </c>
@@ -11539,7 +11539,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="151" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A151" s="2" t="s">
         <v>115</v>
       </c>
@@ -11610,7 +11610,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="152" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A152" s="2" t="s">
         <v>115</v>
       </c>
@@ -11681,7 +11681,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="153" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A153" s="2" t="s">
         <v>115</v>
       </c>
@@ -11752,7 +11752,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="154" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A154" s="2" t="s">
         <v>115</v>
       </c>
@@ -11823,7 +11823,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="155" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A155" s="2" t="s">
         <v>115</v>
       </c>
@@ -11894,7 +11894,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="156" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A156" s="2" t="s">
         <v>115</v>
       </c>
@@ -11965,7 +11965,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="157" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A157" s="2" t="s">
         <v>115</v>
       </c>
@@ -12036,7 +12036,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="158" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A158" s="2" t="s">
         <v>115</v>
       </c>
@@ -12107,7 +12107,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="159" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A159" s="2" t="s">
         <v>115</v>
       </c>
@@ -12178,7 +12178,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="160" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A160" s="2" t="s">
         <v>115</v>
       </c>
@@ -12249,7 +12249,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="161" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A161" s="2" t="s">
         <v>115</v>
       </c>
@@ -12320,7 +12320,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="162" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A162" s="2" t="s">
         <v>115</v>
       </c>
@@ -12391,7 +12391,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="163" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A163" s="2" t="s">
         <v>115</v>
       </c>
@@ -12462,7 +12462,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="164" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A164" s="2" t="s">
         <v>115</v>
       </c>
@@ -12533,7 +12533,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="165" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A165" s="2" t="s">
         <v>115</v>
       </c>
@@ -12604,7 +12604,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="166" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A166" s="2" t="s">
         <v>115</v>
       </c>
@@ -12675,7 +12675,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="167" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A167" s="2" t="s">
         <v>115</v>
       </c>
@@ -12746,7 +12746,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="168" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A168" s="2" t="s">
         <v>115</v>
       </c>
@@ -12817,7 +12817,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="169" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A169" s="2" t="s">
         <v>115</v>
       </c>
@@ -12888,7 +12888,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="170" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A170" s="2" t="s">
         <v>115</v>
       </c>
@@ -12959,7 +12959,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="171" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A171" s="2" t="s">
         <v>115</v>
       </c>
@@ -13030,7 +13030,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="172" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A172" s="2" t="s">
         <v>115</v>
       </c>
@@ -13101,7 +13101,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="173" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A173" s="2" t="s">
         <v>115</v>
       </c>
@@ -13172,7 +13172,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="174" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A174" s="2" t="s">
         <v>115</v>
       </c>
@@ -13243,7 +13243,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="175" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A175" s="2" t="s">
         <v>115</v>
       </c>
@@ -13314,7 +13314,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="176" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A176" s="2" t="s">
         <v>115</v>
       </c>
@@ -13385,7 +13385,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="177" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A177" s="2" t="s">
         <v>115</v>
       </c>
@@ -13456,7 +13456,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="178" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A178" s="2" t="s">
         <v>115</v>
       </c>
@@ -13527,7 +13527,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="179" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A179" s="2" t="s">
         <v>115</v>
       </c>
@@ -13598,7 +13598,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="180" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A180" s="2" t="s">
         <v>115</v>
       </c>
@@ -13669,7 +13669,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="181" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A181" s="2" t="s">
         <v>115</v>
       </c>
@@ -13740,7 +13740,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="182" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A182" s="2" t="s">
         <v>115</v>
       </c>
@@ -13811,7 +13811,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="183" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A183" s="2" t="s">
         <v>115</v>
       </c>
@@ -13882,7 +13882,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="184" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A184" s="2" t="s">
         <v>115</v>
       </c>
@@ -13953,7 +13953,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="185" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A185" s="2" t="s">
         <v>115</v>
       </c>
@@ -14024,7 +14024,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="186" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A186" s="2" t="s">
         <v>115</v>
       </c>
@@ -14095,7 +14095,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="187" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A187" s="2" t="s">
         <v>115</v>
       </c>
@@ -14166,7 +14166,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="188" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A188" s="2" t="s">
         <v>115</v>
       </c>
@@ -14237,7 +14237,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="189" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A189" s="2" t="s">
         <v>115</v>
       </c>
@@ -14308,7 +14308,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="190" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A190" s="2" t="s">
         <v>115</v>
       </c>
@@ -14379,7 +14379,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="191" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A191" s="2" t="s">
         <v>115</v>
       </c>
@@ -14450,7 +14450,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="192" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A192" s="2" t="s">
         <v>115</v>
       </c>
@@ -14521,7 +14521,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="193" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A193" s="2" t="s">
         <v>115</v>
       </c>
@@ -14592,7 +14592,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="194" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A194" s="2" t="s">
         <v>115</v>
       </c>
@@ -14663,7 +14663,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="195" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A195" s="2" t="s">
         <v>115</v>
       </c>
@@ -14734,7 +14734,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="196" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A196" s="2" t="s">
         <v>115</v>
       </c>
@@ -14805,7 +14805,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="197" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A197" s="2" t="s">
         <v>115</v>
       </c>
@@ -14876,7 +14876,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="198" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A198" s="2" t="s">
         <v>115</v>
       </c>
@@ -14947,7 +14947,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="199" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A199" s="2" t="s">
         <v>115</v>
       </c>
@@ -15018,7 +15018,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="200" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A200" s="2" t="s">
         <v>115</v>
       </c>
@@ -15089,7 +15089,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="201" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A201" s="2" t="s">
         <v>115</v>
       </c>
@@ -15160,7 +15160,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="202" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A202" s="2" t="s">
         <v>115</v>
       </c>
@@ -15231,7 +15231,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="203" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A203" s="2" t="s">
         <v>115</v>
       </c>
@@ -15302,7 +15302,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="204" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A204" s="2" t="s">
         <v>115</v>
       </c>
@@ -15373,7 +15373,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="205" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A205" s="2" t="s">
         <v>115</v>
       </c>
@@ -15444,7 +15444,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="206" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A206" s="2" t="s">
         <v>115</v>
       </c>
@@ -15515,7 +15515,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="207" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A207" s="2" t="s">
         <v>115</v>
       </c>
@@ -15586,7 +15586,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="208" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A208" s="2" t="s">
         <v>115</v>
       </c>
@@ -15657,7 +15657,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="209" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A209" s="2" t="s">
         <v>115</v>
       </c>
@@ -15728,7 +15728,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="210" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A210" s="2" t="s">
         <v>115</v>
       </c>
@@ -15799,7 +15799,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="211" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A211" s="2" t="s">
         <v>115</v>
       </c>
@@ -15870,7 +15870,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="212" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A212" s="2" t="s">
         <v>115</v>
       </c>
@@ -15941,7 +15941,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="213" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A213" s="2" t="s">
         <v>115</v>
       </c>
@@ -16012,7 +16012,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="214" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A214" s="2" t="s">
         <v>115</v>
       </c>
@@ -16083,7 +16083,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="215" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A215" s="2" t="s">
         <v>115</v>
       </c>
@@ -16155,7 +16155,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:W2" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>